<commit_message>
fix music-analysis groundtruth cutoff
</commit_message>
<xml_diff>
--- a/tasks/finalpool/music-analysis/groundtruth_workspace/music_analysis_result.xlsx
+++ b/tasks/finalpool/music-analysis/groundtruth_workspace/music_analysis_result.xlsx
@@ -9055,7 +9055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9701,54 +9701,50 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Blues in the Night</t>
+          <t>Deep in the Heart of Texas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Woody Herman &amp; His Orchestra</t>
+          <t>Alvino Rey &amp; His Orchestra with Bill Schallen &amp; Skeets Herfurt</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Weeks 2-2</t>
+          <t>Weeks 3-3</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Weeks 2-2</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Deep in the Heart of Texas</t>
+          <t>Der Fuehrer's Face</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alvino Rey &amp; His Orchestra with Bill Schallen &amp; Skeets Herfurt</t>
+          <t>Spike Jones &amp; His City Slickers with Carl Grayson</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
         <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Weeks 3-3</t>
+          <t>Weeks 4-4</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -9759,23 +9755,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Der Fuehrer's Face</t>
+          <t>I Had the Craziest Dream</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Spike Jones &amp; His City Slickers with Carl Grayson</t>
+          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Weeks 4-4</t>
+          <t>Weeks 6-6</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -9786,23 +9782,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Der Fuehrer's Face</t>
+          <t>I Left My Heart at the Stage Door Canteen</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Spike Jones &amp; His City Slickers with Carl Grayson</t>
+          <t>Sammy Kaye &amp; His Orchestra with Don Cornell</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
         <v>1</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Weeks 2-2</t>
+          <t>Weeks 3-3</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -9813,23 +9809,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>I Had the Craziest Dream</t>
+          <t>I Said No!</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
+          <t>Alvino Rey &amp; His Orchestra with Yvonne King</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D27" t="n">
         <v>1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Weeks 6-6</t>
+          <t>Weeks 4-4</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -9840,23 +9836,23 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>I Left My Heart at the Stage Door Canteen</t>
+          <t>Just as Though You Were Here</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sammy Kaye &amp; His Orchestra with Don Cornell</t>
+          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra and The Pied Pipers</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Weeks 3-3</t>
+          <t>Weeks 8-8</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -9867,16 +9863,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>I Said No!</t>
+          <t>Mister Five by Five</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alvino Rey &amp; His Orchestra with Yvonne King</t>
+          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
@@ -9894,23 +9890,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>I Said No!</t>
+          <t>Piano Concerto in B Flat</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alvino Rey &amp; His Orchestra with Yvonne King</t>
+          <t>Freddy Martin &amp; His Orchestra with Jack Fina</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
         <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Weeks 2-2</t>
+          <t>Weeks 1-1</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -9921,23 +9917,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Just as Though You Were Here</t>
+          <t>Remember Pearl Harbor</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra and The Pied Pipers</t>
+          <t>Sammy Kaye &amp; His Orchestra with The Glee Club</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Weeks 8-8</t>
+          <t>Weeks 3-3</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -9948,23 +9944,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mister Five by Five</t>
+          <t>When the Lights Go On Again (All Over the World)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
+          <t>Vaughn Monroe &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Weeks 4-4</t>
+          <t>Weeks 7-7</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -9975,25 +9971,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Piano Concerto in B Flat</t>
+          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Freddy Martin &amp; His Orchestra with Jack Fina</t>
+          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Weeks 1-1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
         <v>0</v>
       </c>
@@ -10002,25 +9994,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Remember Pearl Harbor</t>
+          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sammy Kaye &amp; His Orchestra with The Glee Club</t>
+          <t>Kate Smith</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Weeks 3-3</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
         <v>0</v>
       </c>
@@ -10029,25 +10017,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Serenade in Blue</t>
+          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; The Modernaires</t>
+          <t>Kay Kyser &amp; His Orchestra with Harry Babbit &amp; The Glee Club</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Weeks 2-2</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
         <v>0</v>
       </c>
@@ -10056,25 +10040,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>When the Lights Go On Again (All Over the World)</t>
+          <t>A Zoot Suit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vaughn Monroe &amp; His Orchestra</t>
+          <t>Kay Kyser &amp; His Orchestra with Sully Mason &amp; Trudy Erwin</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Weeks 7-7</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
         <v>0</v>
       </c>
@@ -10083,16 +10063,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>(I've Got a Gal In) Kalamazoo</t>
+          <t>Always on my Heart</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Marion Hutton &amp; Tex Beneke</t>
+          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -10106,16 +10086,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
+          <t>Amen</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
+          <t>Abe Lyman &amp; His Orchestra &amp; Chorus with Rose Blane</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -10129,16 +10109,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
+          <t>Amen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Kate Smith</t>
+          <t>Woody Herman &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -10152,12 +10132,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>(There'll Be Bluebirds Over) The White Cliffs of Dover</t>
+          <t>Blues in the Night</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with Harry Babbit &amp; The Glee Club</t>
+          <t>Cab Calloway</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -10175,16 +10155,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>A String of Pearls</t>
+          <t>Blues in the Night</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra</t>
+          <t>Dinah Shore</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -10198,16 +10178,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>A Zoot Suit</t>
+          <t>Blues in the Night</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with Sully Mason &amp; Trudy Erwin</t>
+          <t>Jimmy Lunceford &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -10221,16 +10201,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Always on my Heart</t>
+          <t>Cow-Cow Boogie</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
+          <t>Freddie Slack &amp; His Orchestra with Ella Mae Morse</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -10244,12 +10224,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Amen</t>
+          <t>Daybreak</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Abe Lyman &amp; His Orchestra &amp; Chorus with Rose Blane</t>
+          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -10267,16 +10247,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Amen</t>
+          <t>Dearly Beloved</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Woody Herman &amp; His Orchestra</t>
+          <t>Dinah Shore</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -10290,16 +10270,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Blues in the Night</t>
+          <t>Dearly Beloved</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cab Calloway</t>
+          <t>Glenn Miller &amp; His Orchestra with Skip Nelson</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -10313,16 +10293,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Blues in the Night</t>
+          <t>Deep in the Heart of Texas</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dinah Shore</t>
+          <t>Horace Heidt &amp; His Musical Knights</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
@@ -10336,16 +10316,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Blues in the Night</t>
+          <t>Everything I Love</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jimmy Lunceford &amp; His Orchestra</t>
+          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; Chorus</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -10359,16 +10339,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Chatanooga Choo Choo</t>
+          <t>He's My Guy</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Tex Beneke &amp; The Modernaires</t>
+          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -10382,16 +10362,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cow-Cow Boogie</t>
+          <t>I Don't Want to Talk Without You</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Freddie Slack &amp; His Orchestra with Ella Mae Morse</t>
+          <t>Bing Crosby</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -10405,12 +10385,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Daybreak</t>
+          <t>I Left My Heart at the Stage Door Canteen</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra</t>
+          <t>Charlie Spivak &amp; His Orchestra with Garry Stevens</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -10428,12 +10408,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dearly Beloved</t>
+          <t>I Remember You</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dinah Shore</t>
+          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -10451,16 +10431,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dearly Beloved</t>
+          <t>I Said No</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Skip Nelson</t>
+          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly &amp; Helen O'Connell</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -10474,12 +10454,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Deep in the Heart of Texas</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Horace Heidt &amp; His Musical Knights</t>
+          <t>Benny Goodman &amp; His Orchestra with Dick Haymes</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -10497,16 +10477,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Don't Sit Under the Apple Tree</t>
+          <t>Jersey Bounce</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Marion Hutton &amp; Tex Beneke</t>
+          <t>Jimmy Dorsey &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -10520,16 +10500,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Everything I Love</t>
+          <t>Jingle, Jangle, Jingle</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; Chorus</t>
+          <t>The Merry Macs</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -10543,16 +10523,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>He Wears a Pair of Silver Wings</t>
+          <t>Johnny Doughboy Found a Rose in Ireland</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with Harry Babbitt</t>
+          <t>Guy Lombardo &amp; His Royal Canadians with Kenny Gardner</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -10566,12 +10546,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>He's My Guy</t>
+          <t>Johnny Doughboy Found a Rose in Ireland</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
+          <t>Kay Kyser &amp; His Orchestra with The Glee Cliub</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -10589,16 +10569,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>I Don't Want to Talk Without You</t>
+          <t>Juke Box Saturday Night</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Bing Crosby</t>
+          <t>Glenn Miller &amp; His Orchestra with Tex Beneke &amp; Marion Hutton</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -10612,7 +10592,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>I Don't Want to Walk Without You</t>
+          <t>Manhattan Serenade</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10621,7 +10601,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -10635,12 +10615,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>I Left My Heart at the Stage Door Canteen</t>
+          <t>Miss You</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Charlie Spivak &amp; His Orchestra with Garry Stevens</t>
+          <t>Bing Crosby</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -10658,16 +10638,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>I Remember You</t>
+          <t>Miss You</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly</t>
+          <t>Dinah Shore</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -10681,12 +10661,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>I Said No</t>
+          <t>Mister Five by Five</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly &amp; Helen O'Connell</t>
+          <t>Freddie Slack &amp; His Orchestra with Ella Mae Morse</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -10704,16 +10684,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>Moonlight Becomes You</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Benny Goodman &amp; His Orchestra with Dick Haymes</t>
+          <t>Glenn Miller &amp; His Orchestra with Skip Nelson &amp; The Modernaires</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -10727,16 +10707,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jersey Bounce</t>
+          <t>My Devotion</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Benny Goodman &amp; His Orchestra</t>
+          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -10750,16 +10730,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Jersey Bounce</t>
+          <t>My Devotion</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jimmy Dorsey &amp; His Orchestra</t>
+          <t>Vaughn Monroe &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -10773,16 +10753,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Jingle, Jangle, Jingle</t>
+          <t>One Dozen Roses</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with Harry Babbitt &amp; Julie Conway</t>
+          <t>Dinah Shore</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -10796,16 +10776,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Jingle, Jangle, Jingle</t>
+          <t>One Dozen Roses</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>The Merry Macs</t>
+          <t>Glen Gray &amp; The Casa Loma Orchestra with Pee Wee Hunt</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -10819,16 +10799,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Johnny Doughboy Found a Rose in Ireland</t>
+          <t>One Dozen Roses</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Guy Lombardo &amp; His Royal Canadians with Kenny Gardner</t>
+          <t>Harry James &amp; His Music Masters with Jimmy Saunders</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -10842,16 +10822,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Johnny Doughboy Found a Rose in Ireland</t>
+          <t>Praise the Lord and Pass the Ammunition</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with The Glee Cliub</t>
+          <t>The Merry Macs</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -10865,16 +10845,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Juke Box Saturday Night</t>
+          <t>Rosie O'Day (The Filla-Ga-Dusha Song)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Tex Beneke &amp; Marion Hutton</t>
+          <t>Kate Smith</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -10888,16 +10868,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Manhattan Serenade</t>
+          <t>Shepherd Serenade</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Makers with Hellen Forrest</t>
+          <t>Bing Crosby</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -10911,16 +10891,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Miss You</t>
+          <t>Skylark</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Bing Crosby</t>
+          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -10934,16 +10914,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Miss You</t>
+          <t>Somebody Else Is Taking My Place</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dinah Shore</t>
+          <t>Benny Goodman &amp; His Orchestra with Peggy Lee</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -10957,16 +10937,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Mister Five by Five</t>
+          <t>Somebody Else Is Taking My Place</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Freddie Slack &amp; His Orchestra with Ella Mae Morse</t>
+          <t>Russ Morgan &amp; His Orchestra with The Morganaires</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
@@ -10980,16 +10960,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Moonlight Becomes You</t>
+          <t>Strictly Instrumental</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Skip Nelson &amp; The Modernaires</t>
+          <t>Harry James &amp; His Music Makers</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -11003,16 +10983,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Moonlight Cocktail</t>
+          <t>Strip Polka</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; The Modernaires</t>
+          <t>Alvino Rey &amp; His Orchestra &amp; His Chorus with The Four King Sisters</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -11026,16 +11006,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>My Devotion</t>
+          <t>Strip Polka</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Charlie Spivak &amp; His Orchestra with Garry Stevens</t>
+          <t>Johnny Mercer &amp; The Mellowaires</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -11049,16 +11029,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>My Devotion</t>
+          <t>Strip Polka</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly</t>
+          <t>Kay Kyser &amp; His Orchestra with Jack Martin &amp; The Glee Club</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -11072,16 +11052,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>My Devotion</t>
+          <t>Strip Polka</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Vaughn Monroe &amp; His Orchestra</t>
+          <t>The Andrews Sister</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -11095,16 +11075,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>One Dozen Roses</t>
+          <t>Sweet Eloise</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Dinah Shore</t>
+          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; The Modernaires</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -11118,16 +11098,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>One Dozen Roses</t>
+          <t>Take Me</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Glen Gray &amp; The Casa Loma Orchestra with Pee Wee Hunt</t>
+          <t>Benny Goodman &amp; His Orchestra with Dick Haymes</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -11141,16 +11121,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>One Dozen Roses</t>
+          <t>Take Me</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Masters with Jimmy Saunders</t>
+          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -11164,16 +11144,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>One Dozen Roses</t>
+          <t>This is No Laughing Matter</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Harry James &amp; His Music Masters with Jimmy Saunders</t>
+          <t>Charlie Spivak &amp; His Orchestra with Garry Stevens</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -11187,16 +11167,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Praise the Lord and Pass the Ammunition</t>
+          <t>Tonight We Love</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Kay Kyser &amp; His Orchestra with The Glee Cliub</t>
+          <t>Tony Martin with David Rose &amp; His Orchestra</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -11210,16 +11190,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Praise the Lord and Pass the Ammunition</t>
+          <t>Why Don't You Do Right?</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>The Merry Macs</t>
+          <t>Benny Goodman and His Orchestra</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -11233,12 +11213,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Rosie O'Day (The Filla-Ga-Dusha Song)</t>
+          <t>You Made Me Love You</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Kate Smith</t>
+          <t>Harry James &amp; His Music Makers</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -11252,466 +11232,6 @@
         <v>0</v>
       </c>
       <c r="G87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Shepherd Serenade</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Bing Crosby</t>
-        </is>
-      </c>
-      <c r="C88" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" t="n">
-        <v>0</v>
-      </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="n">
-        <v>0</v>
-      </c>
-      <c r="G88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Skylark</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle</t>
-        </is>
-      </c>
-      <c r="C89" t="n">
-        <v>11</v>
-      </c>
-      <c r="D89" t="n">
-        <v>0</v>
-      </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="n">
-        <v>0</v>
-      </c>
-      <c r="G89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Sleepy Lagoon</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Harry James &amp; His Music Makers</t>
-        </is>
-      </c>
-      <c r="C90" t="n">
-        <v>0</v>
-      </c>
-      <c r="D90" t="n">
-        <v>0</v>
-      </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="n">
-        <v>0</v>
-      </c>
-      <c r="G90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Somebody Else Is Taking My Place</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Benny Goodman &amp; His Orchestra with Peggy Lee</t>
-        </is>
-      </c>
-      <c r="C91" t="n">
-        <v>9</v>
-      </c>
-      <c r="D91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Somebody Else Is Taking My Place</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Russ Morgan &amp; His Orchestra with The Morganaires</t>
-        </is>
-      </c>
-      <c r="C92" t="n">
-        <v>6</v>
-      </c>
-      <c r="D92" t="n">
-        <v>0</v>
-      </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G92" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Strictly Instrumental</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Harry James &amp; His Music Makers</t>
-        </is>
-      </c>
-      <c r="C93" t="n">
-        <v>4</v>
-      </c>
-      <c r="D93" t="n">
-        <v>0</v>
-      </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="n">
-        <v>0</v>
-      </c>
-      <c r="G93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Strip Polka</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Alvino Rey &amp; His Orchestra &amp; His Chorus with The Four King Sisters</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>2</v>
-      </c>
-      <c r="D94" t="n">
-        <v>0</v>
-      </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="n">
-        <v>0</v>
-      </c>
-      <c r="G94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Strip Polka</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Johnny Mercer &amp; The Mellowaires</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>3</v>
-      </c>
-      <c r="D95" t="n">
-        <v>0</v>
-      </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="n">
-        <v>0</v>
-      </c>
-      <c r="G95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Strip Polka</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Kay Kyser &amp; His Orchestra with Jack Martin &amp; The Glee Club</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Strip Polka</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>The Andrews Sister</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>4</v>
-      </c>
-      <c r="D97" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="n">
-        <v>0</v>
-      </c>
-      <c r="G97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Sweet Eloise</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Glenn Miller &amp; His Orchestra with Ray Eberle &amp; The Modernaires</t>
-        </is>
-      </c>
-      <c r="C98" t="n">
-        <v>3</v>
-      </c>
-      <c r="D98" t="n">
-        <v>0</v>
-      </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="n">
-        <v>0</v>
-      </c>
-      <c r="G98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Take Me</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Benny Goodman &amp; His Orchestra with Dick Haymes</t>
-        </is>
-      </c>
-      <c r="C99" t="n">
-        <v>1</v>
-      </c>
-      <c r="D99" t="n">
-        <v>0</v>
-      </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Take Me</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Tommy Dorsey &amp; His Orchestra with Frank Sinatra</t>
-        </is>
-      </c>
-      <c r="C100" t="n">
-        <v>3</v>
-      </c>
-      <c r="D100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Tangerine</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Jimmy Dorsey &amp; His Orchestra with Bob Eberly &amp; Helen O'Connell</t>
-        </is>
-      </c>
-      <c r="C101" t="n">
-        <v>0</v>
-      </c>
-      <c r="D101" t="n">
-        <v>0</v>
-      </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>This is No Laughing Matter</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Charlie Spivak &amp; His Orchestra with Garry Stevens</t>
-        </is>
-      </c>
-      <c r="C102" t="n">
-        <v>1</v>
-      </c>
-      <c r="D102" t="n">
-        <v>0</v>
-      </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Tonight We Love</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Tony Martin with David Rose &amp; His Orchestra</t>
-        </is>
-      </c>
-      <c r="C103" t="n">
-        <v>1</v>
-      </c>
-      <c r="D103" t="n">
-        <v>0</v>
-      </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="n">
-        <v>0</v>
-      </c>
-      <c r="G103" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>White Christmas</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Bing Crosby &amp; The Ken Darby Singers with John Scott Trotter</t>
-        </is>
-      </c>
-      <c r="C104" t="n">
-        <v>0</v>
-      </c>
-      <c r="D104" t="n">
-        <v>0</v>
-      </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Who Wouldn't Love You</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Kay Kyser &amp; His Orchestra with Harry Babbit &amp; Trudy Erwin</t>
-        </is>
-      </c>
-      <c r="C105" t="n">
-        <v>0</v>
-      </c>
-      <c r="D105" t="n">
-        <v>0</v>
-      </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Why Don't You Do Right?</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Benny Goodman and His Orchestra</t>
-        </is>
-      </c>
-      <c r="C106" t="n">
-        <v>1</v>
-      </c>
-      <c r="D106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>You Made Me Love You</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Harry James &amp; His Music Makers</t>
-        </is>
-      </c>
-      <c r="C107" t="n">
-        <v>3</v>
-      </c>
-      <c r="D107" t="n">
-        <v>0</v>
-      </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>